<commit_message>
Flag possible dual role of pensamiento del profesor: Dim.2 and Dim.5
Investigator's instinct that Feldman/Cols might serve Dimensión 5 (diseño
didáctico), not just the representaciones/concepciones debate in Dimensión
2, has real grounding: Jackson's preactive phase is specifically about
planning/design decisions. Added a note to the ficha so both angles get
checked while reading, rather than deciding now without having read the
texts.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -458,6 +458,13 @@
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Estado: Cabello/Aprea (2006) está completo, con cita textual ya confirmada contra la introducción que compartiste. Los demás (Feldman 1995, Cols 2000, Cols 2011, Montenegro et al. 1996, Machicado 2022 como antecedente metodológico) son andamiajes -- las preguntas ya apuntadas a tu corpus, para que los completes al leer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Actualización 2026-10-17: al leer Feldman y Cols, prestar atención a DOS preguntas, no una sola -- (1) la original, representaciones vs. concepciones docentes para la Dimensión 2; y (2) si el texto habla específicamente de la fase PREACTIVA (planificación, antes de dar la clase, en términos de Jackson) -- de ser así, el texto puede servir también para la Dimensión 5 (diseño didáctico), en diálogo con Palamidessi y Gvirtz (1998), que es el anclaje ya fijado de esa dimensión. No es necesariamente una cosa o la otra -- un mismo texto puede aportar a las dos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep pensamiento del profesor ficha scoped to Dimensión 2 only
Investigator prefers not to mix the representaciones/concepciones
question (Dim.2) with diseño didáctico observations (Dim.5) in the same
ficha. Revised the previous note accordingly.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
@@ -461,10 +461,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="50" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Actualización 2026-10-17: al leer Feldman y Cols, prestar atención a DOS preguntas, no una sola -- (1) la original, representaciones vs. concepciones docentes para la Dimensión 2; y (2) si el texto habla específicamente de la fase PREACTIVA (planificación, antes de dar la clase, en términos de Jackson) -- de ser así, el texto puede servir también para la Dimensión 5 (diseño didáctico), en diálogo con Palamidessi y Gvirtz (1998), que es el anclaje ya fijado de esa dimensión. No es necesariamente una cosa o la otra -- un mismo texto puede aportar a las dos.</t>
+          <t>Actualización 2026-10-17 (revisada): al leer Feldman y Cols, esta ficha sigue siendo solo para la discusión representaciones vs. concepciones docentes (Dimensión 2). Si algo del texto habla específicamente de la fase PREACTIVA (planificación, antes de dar la clase) y podría servir para Dimensión 5 (diseño didáctico, junto a Palamidessi y Gvirtz), anotalo aparte, no acá -- la investigadora prefiere no mezclar las dos cosas en la misma ficha.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix misreading of "ficha aparte": no file split needed after all
The investigator meant fichas_lectura_pensamiento_profesor.xlsx is
already the separate ficha (apart from representaciones_sociales), not
that Dim.2/Dim.5 observations needed splitting within it. Reverted the
previous scoping note back to tracking both questions in this one ficha.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
@@ -461,10 +461,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Actualización 2026-10-17 (revisada): al leer Feldman y Cols, esta ficha sigue siendo solo para la discusión representaciones vs. concepciones docentes (Dimensión 2). Si algo del texto habla específicamente de la fase PREACTIVA (planificación, antes de dar la clase) y podría servir para Dimensión 5 (diseño didáctico, junto a Palamidessi y Gvirtz), anotalo aparte, no acá -- la investigadora prefiere no mezclar las dos cosas en la misma ficha.</t>
+          <t>Actualización 2026-10-17: al leer Feldman y Cols, prestar atención a DOS preguntas, no una sola -- (1) la original, representaciones vs. concepciones docentes para la Dimensión 2; y (2) si el texto habla específicamente de la fase PREACTIVA (planificación, antes de dar la clase, en términos de Jackson) -- de ser así, el texto puede servir también para la Dimensión 5 (diseño didáctico), en diálogo con Palamidessi y Gvirtz (1998), que es el anclaje ya fijado de esa dimensión. Ambas preguntas se registran en esta misma ficha (pensamiento del profesor), que ya está separada de la de representaciones sociales -- no hace falta un archivo nuevo por dimensión.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-point pensamiento del profesor ficha: representaciones→acciones, not diseño didáctico
Investigator's reconsideration while reading Feldman/Cols is stronger than the
10/17 hypothesis: 1.6 is already covered by the newly-verified Gvirtz & Palamidessi
citation, so the real contribution would be an independent theoretical confirmation
of the representations-condition-practice argument already carried by Aprea/Cabello,
feeding 1.1 instead. Updated the ficha's reading question accordingly.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_pensamiento_profesor.xlsx
@@ -461,10 +461,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="75" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Actualización 2026-10-17: al leer Feldman y Cols, prestar atención a DOS preguntas, no una sola -- (1) la original, representaciones vs. concepciones docentes para la Dimensión 2; y (2) si el texto habla específicamente de la fase PREACTIVA (planificación, antes de dar la clase, en términos de Jackson) -- de ser así, el texto puede servir también para la Dimensión 5 (diseño didáctico), en diálogo con Palamidessi y Gvirtz (1998), que es el anclaje ya fijado de esa dimensión. Ambas preguntas se registran en esta misma ficha (pensamiento del profesor), que ya está separada de la de representaciones sociales -- no hace falta un archivo nuevo por dimensión.</t>
+          <t>Actualización 2026-10-29 (revisada otra vez): al leer Feldman y Cols, la pregunta principal ya NO es si sirven para Dimensión 5/diseño didáctico (esa ya está cubierta por Gvirtz y Palamidessi, 1998, con cita textual verificada). La pregunta principal es si sostienen, desde otra tradición teórica (teorías personales/repertorios sociales), el mismo argumento central de esta tesis: que las representaciones condicionan las prácticas concretas de enseñanza -- el mismo argumento que ya sostiene Aprea/Cabello desde la TRS. Si es así, van al apartado 1.1 del Marco Teórico (representaciones sociales) como una segunda confirmación teórica independiente, no a 1.6. Buscar específicamente pasajes sobre cómo las 'teorías personales' o 'repertorios' de las docentes se traducen en decisiones concretas de enseñanza. La pista de la fase preactiva (Jackson, nota anterior) queda como posibilidad secundaria, no descartada pero no prioritaria.</t>
         </is>
       </c>
     </row>

</xml_diff>